<commit_message>
Add Excel equipment master and clarify selected calendar dates
</commit_message>
<xml_diff>
--- a/member-registration.xlsx
+++ b/member-registration.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="会員登録" sheetId="1" r:id="Ra700e3b5ddc840e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入力方法" sheetId="2" r:id="Rd710b11fddc64f1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="会員登録" sheetId="1" r:id="R0df375ad67ab4a60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入力方法" sheetId="2" r:id="R3e242ebad94a4c20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="備品マスター" sheetId="3" r:id="R6abe4763f8e54cba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +18,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="@"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -36,6 +37,12 @@
       <x:b/>
       <x:sz val="15"/>
       <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
   <x:fills count="5">
@@ -67,7 +74,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="13">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -83,6 +90,10 @@
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1999,4 +2010,559 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="10" t="str">
+        <x:v>操作</x:v>
+      </x:c>
+      <x:c r="B1" s="10" t="str">
+        <x:v>備品ID</x:v>
+      </x:c>
+      <x:c r="C1" s="10" t="str">
+        <x:v>備品名</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="12" t="str">
+        <x:v>登録・更新</x:v>
+      </x:c>
+      <x:c r="B2" s="12" t="str">
+        <x:v>equipment1</x:v>
+      </x:c>
+      <x:c r="C2" s="12" t="str">
+        <x:v>ボールケース</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="A3" s="12" t="str">
+        <x:v>登録・更新</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
+        <x:v>equipment2</x:v>
+      </x:c>
+      <x:c r="C3" s="12" t="str">
+        <x:v>救急箱</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="12" t="str">
+        <x:v>登録・更新</x:v>
+      </x:c>
+      <x:c r="B4" s="12" t="str">
+        <x:v>equipment3</x:v>
+      </x:c>
+      <x:c r="C4" s="12" t="str">
+        <x:v>タイマー</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="28" customHeight="1">
+      <x:c r="A5" s="12" t="str">
+        <x:v>登録・更新</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="str">
+        <x:v>equipment4</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="str">
+        <x:v>作戦板</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="28" customHeight="1">
+      <x:c r="A6" s="12" t="str">
+        <x:v>登録・更新</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="str">
+        <x:v>equipment5</x:v>
+      </x:c>
+      <x:c r="C6" s="12" t="str">
+        <x:v>ユニフォーム</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="28" customHeight="1">
+      <x:c r="A7" s="12"/>
+      <x:c r="B7" s="12"/>
+      <x:c r="C7" s="12"/>
+    </x:row>
+    <x:row r="8" ht="28" customHeight="1">
+      <x:c r="A8" s="12"/>
+      <x:c r="B8" s="12"/>
+      <x:c r="C8" s="12"/>
+    </x:row>
+    <x:row r="9" ht="28" customHeight="1">
+      <x:c r="A9" s="12"/>
+      <x:c r="B9" s="12"/>
+      <x:c r="C9" s="12"/>
+    </x:row>
+    <x:row r="10" ht="28" customHeight="1">
+      <x:c r="A10" s="12"/>
+      <x:c r="B10" s="12"/>
+      <x:c r="C10" s="12"/>
+    </x:row>
+    <x:row r="11" ht="28" customHeight="1">
+      <x:c r="A11" s="12"/>
+      <x:c r="B11" s="12"/>
+      <x:c r="C11" s="12"/>
+    </x:row>
+    <x:row r="12" ht="28" customHeight="1">
+      <x:c r="A12" s="12"/>
+      <x:c r="B12" s="12"/>
+      <x:c r="C12" s="12"/>
+    </x:row>
+    <x:row r="13" ht="28" customHeight="1">
+      <x:c r="A13" s="12"/>
+      <x:c r="B13" s="12"/>
+      <x:c r="C13" s="12"/>
+    </x:row>
+    <x:row r="14" ht="28" customHeight="1">
+      <x:c r="A14" s="12"/>
+      <x:c r="B14" s="12"/>
+      <x:c r="C14" s="12"/>
+    </x:row>
+    <x:row r="15" ht="28" customHeight="1">
+      <x:c r="A15" s="12"/>
+      <x:c r="B15" s="12"/>
+      <x:c r="C15" s="12"/>
+    </x:row>
+    <x:row r="16" ht="28" customHeight="1">
+      <x:c r="A16" s="12"/>
+      <x:c r="B16" s="12"/>
+      <x:c r="C16" s="12"/>
+    </x:row>
+    <x:row r="17" ht="28" customHeight="1">
+      <x:c r="A17" s="12"/>
+      <x:c r="B17" s="12"/>
+      <x:c r="C17" s="12"/>
+    </x:row>
+    <x:row r="18" ht="28" customHeight="1">
+      <x:c r="A18" s="12"/>
+      <x:c r="B18" s="12"/>
+      <x:c r="C18" s="12"/>
+    </x:row>
+    <x:row r="19" ht="28" customHeight="1">
+      <x:c r="A19" s="12"/>
+      <x:c r="B19" s="12"/>
+      <x:c r="C19" s="12"/>
+    </x:row>
+    <x:row r="20" ht="28" customHeight="1">
+      <x:c r="A20" s="12"/>
+      <x:c r="B20" s="12"/>
+      <x:c r="C20" s="12"/>
+    </x:row>
+    <x:row r="21" ht="28" customHeight="1">
+      <x:c r="A21" s="12"/>
+      <x:c r="B21" s="12"/>
+      <x:c r="C21" s="12"/>
+    </x:row>
+    <x:row r="22" ht="28" customHeight="1">
+      <x:c r="A22" s="12"/>
+      <x:c r="B22" s="12"/>
+      <x:c r="C22" s="12"/>
+    </x:row>
+    <x:row r="23" ht="28" customHeight="1">
+      <x:c r="A23" s="12"/>
+      <x:c r="B23" s="12"/>
+      <x:c r="C23" s="12"/>
+    </x:row>
+    <x:row r="24" ht="28" customHeight="1">
+      <x:c r="A24" s="12"/>
+      <x:c r="B24" s="12"/>
+      <x:c r="C24" s="12"/>
+    </x:row>
+    <x:row r="25" ht="28" customHeight="1">
+      <x:c r="A25" s="12"/>
+      <x:c r="B25" s="12"/>
+      <x:c r="C25" s="12"/>
+    </x:row>
+    <x:row r="26" ht="28" customHeight="1">
+      <x:c r="A26" s="12"/>
+      <x:c r="B26" s="12"/>
+      <x:c r="C26" s="12"/>
+    </x:row>
+    <x:row r="27" ht="28" customHeight="1">
+      <x:c r="A27" s="12"/>
+      <x:c r="B27" s="12"/>
+      <x:c r="C27" s="12"/>
+    </x:row>
+    <x:row r="28" ht="28" customHeight="1">
+      <x:c r="A28" s="12"/>
+      <x:c r="B28" s="12"/>
+      <x:c r="C28" s="12"/>
+    </x:row>
+    <x:row r="29" ht="28" customHeight="1">
+      <x:c r="A29" s="12"/>
+      <x:c r="B29" s="12"/>
+      <x:c r="C29" s="12"/>
+    </x:row>
+    <x:row r="30" ht="28" customHeight="1">
+      <x:c r="A30" s="12"/>
+      <x:c r="B30" s="12"/>
+      <x:c r="C30" s="12"/>
+    </x:row>
+    <x:row r="31" ht="28" customHeight="1">
+      <x:c r="A31" s="12"/>
+      <x:c r="B31" s="12"/>
+      <x:c r="C31" s="12"/>
+    </x:row>
+    <x:row r="32" ht="28" customHeight="1">
+      <x:c r="A32" s="12"/>
+      <x:c r="B32" s="12"/>
+      <x:c r="C32" s="12"/>
+    </x:row>
+    <x:row r="33" ht="28" customHeight="1">
+      <x:c r="A33" s="12"/>
+      <x:c r="B33" s="12"/>
+      <x:c r="C33" s="12"/>
+    </x:row>
+    <x:row r="34" ht="28" customHeight="1">
+      <x:c r="A34" s="12"/>
+      <x:c r="B34" s="12"/>
+      <x:c r="C34" s="12"/>
+    </x:row>
+    <x:row r="35" ht="28" customHeight="1">
+      <x:c r="A35" s="12"/>
+      <x:c r="B35" s="12"/>
+      <x:c r="C35" s="12"/>
+    </x:row>
+    <x:row r="36" ht="28" customHeight="1">
+      <x:c r="A36" s="12"/>
+      <x:c r="B36" s="12"/>
+      <x:c r="C36" s="12"/>
+    </x:row>
+    <x:row r="37" ht="28" customHeight="1">
+      <x:c r="A37" s="12"/>
+      <x:c r="B37" s="12"/>
+      <x:c r="C37" s="12"/>
+    </x:row>
+    <x:row r="38" ht="28" customHeight="1">
+      <x:c r="A38" s="12"/>
+      <x:c r="B38" s="12"/>
+      <x:c r="C38" s="12"/>
+    </x:row>
+    <x:row r="39" ht="28" customHeight="1">
+      <x:c r="A39" s="12"/>
+      <x:c r="B39" s="12"/>
+      <x:c r="C39" s="12"/>
+    </x:row>
+    <x:row r="40" ht="28" customHeight="1">
+      <x:c r="A40" s="12"/>
+      <x:c r="B40" s="12"/>
+      <x:c r="C40" s="12"/>
+    </x:row>
+    <x:row r="41" ht="28" customHeight="1">
+      <x:c r="A41" s="12"/>
+      <x:c r="B41" s="12"/>
+      <x:c r="C41" s="12"/>
+    </x:row>
+    <x:row r="42" ht="28" customHeight="1">
+      <x:c r="A42" s="12"/>
+      <x:c r="B42" s="12"/>
+      <x:c r="C42" s="12"/>
+    </x:row>
+    <x:row r="43" ht="28" customHeight="1">
+      <x:c r="A43" s="12"/>
+      <x:c r="B43" s="12"/>
+      <x:c r="C43" s="12"/>
+    </x:row>
+    <x:row r="44" ht="28" customHeight="1">
+      <x:c r="A44" s="12"/>
+      <x:c r="B44" s="12"/>
+      <x:c r="C44" s="12"/>
+    </x:row>
+    <x:row r="45" ht="28" customHeight="1">
+      <x:c r="A45" s="12"/>
+      <x:c r="B45" s="12"/>
+      <x:c r="C45" s="12"/>
+    </x:row>
+    <x:row r="46" ht="28" customHeight="1">
+      <x:c r="A46" s="12"/>
+      <x:c r="B46" s="12"/>
+      <x:c r="C46" s="12"/>
+    </x:row>
+    <x:row r="47" ht="28" customHeight="1">
+      <x:c r="A47" s="12"/>
+      <x:c r="B47" s="12"/>
+      <x:c r="C47" s="12"/>
+    </x:row>
+    <x:row r="48" ht="28" customHeight="1">
+      <x:c r="A48" s="12"/>
+      <x:c r="B48" s="12"/>
+      <x:c r="C48" s="12"/>
+    </x:row>
+    <x:row r="49" ht="28" customHeight="1">
+      <x:c r="A49" s="12"/>
+      <x:c r="B49" s="12"/>
+      <x:c r="C49" s="12"/>
+    </x:row>
+    <x:row r="50" ht="28" customHeight="1">
+      <x:c r="A50" s="12"/>
+      <x:c r="B50" s="12"/>
+      <x:c r="C50" s="12"/>
+    </x:row>
+    <x:row r="51" ht="28" customHeight="1">
+      <x:c r="A51" s="12"/>
+      <x:c r="B51" s="12"/>
+      <x:c r="C51" s="12"/>
+    </x:row>
+    <x:row r="52" ht="28" customHeight="1">
+      <x:c r="A52" s="12"/>
+      <x:c r="B52" s="12"/>
+      <x:c r="C52" s="12"/>
+    </x:row>
+    <x:row r="53" ht="28" customHeight="1">
+      <x:c r="A53" s="12"/>
+      <x:c r="B53" s="12"/>
+      <x:c r="C53" s="12"/>
+    </x:row>
+    <x:row r="54" ht="28" customHeight="1">
+      <x:c r="A54" s="12"/>
+      <x:c r="B54" s="12"/>
+      <x:c r="C54" s="12"/>
+    </x:row>
+    <x:row r="55" ht="28" customHeight="1">
+      <x:c r="A55" s="12"/>
+      <x:c r="B55" s="12"/>
+      <x:c r="C55" s="12"/>
+    </x:row>
+    <x:row r="56" ht="28" customHeight="1">
+      <x:c r="A56" s="12"/>
+      <x:c r="B56" s="12"/>
+      <x:c r="C56" s="12"/>
+    </x:row>
+    <x:row r="57" ht="28" customHeight="1">
+      <x:c r="A57" s="12"/>
+      <x:c r="B57" s="12"/>
+      <x:c r="C57" s="12"/>
+    </x:row>
+    <x:row r="58" ht="28" customHeight="1">
+      <x:c r="A58" s="12"/>
+      <x:c r="B58" s="12"/>
+      <x:c r="C58" s="12"/>
+    </x:row>
+    <x:row r="59" ht="28" customHeight="1">
+      <x:c r="A59" s="12"/>
+      <x:c r="B59" s="12"/>
+      <x:c r="C59" s="12"/>
+    </x:row>
+    <x:row r="60" ht="28" customHeight="1">
+      <x:c r="A60" s="12"/>
+      <x:c r="B60" s="12"/>
+      <x:c r="C60" s="12"/>
+    </x:row>
+    <x:row r="61" ht="28" customHeight="1">
+      <x:c r="A61" s="12"/>
+      <x:c r="B61" s="12"/>
+      <x:c r="C61" s="12"/>
+    </x:row>
+    <x:row r="62" ht="28" customHeight="1">
+      <x:c r="A62" s="12"/>
+      <x:c r="B62" s="12"/>
+      <x:c r="C62" s="12"/>
+    </x:row>
+    <x:row r="63" ht="28" customHeight="1">
+      <x:c r="A63" s="12"/>
+      <x:c r="B63" s="12"/>
+      <x:c r="C63" s="12"/>
+    </x:row>
+    <x:row r="64" ht="28" customHeight="1">
+      <x:c r="A64" s="12"/>
+      <x:c r="B64" s="12"/>
+      <x:c r="C64" s="12"/>
+    </x:row>
+    <x:row r="65" ht="28" customHeight="1">
+      <x:c r="A65" s="12"/>
+      <x:c r="B65" s="12"/>
+      <x:c r="C65" s="12"/>
+    </x:row>
+    <x:row r="66" ht="28" customHeight="1">
+      <x:c r="A66" s="12"/>
+      <x:c r="B66" s="12"/>
+      <x:c r="C66" s="12"/>
+    </x:row>
+    <x:row r="67" ht="28" customHeight="1">
+      <x:c r="A67" s="12"/>
+      <x:c r="B67" s="12"/>
+      <x:c r="C67" s="12"/>
+    </x:row>
+    <x:row r="68" ht="28" customHeight="1">
+      <x:c r="A68" s="12"/>
+      <x:c r="B68" s="12"/>
+      <x:c r="C68" s="12"/>
+    </x:row>
+    <x:row r="69" ht="28" customHeight="1">
+      <x:c r="A69" s="12"/>
+      <x:c r="B69" s="12"/>
+      <x:c r="C69" s="12"/>
+    </x:row>
+    <x:row r="70" ht="28" customHeight="1">
+      <x:c r="A70" s="12"/>
+      <x:c r="B70" s="12"/>
+      <x:c r="C70" s="12"/>
+    </x:row>
+    <x:row r="71" ht="28" customHeight="1">
+      <x:c r="A71" s="12"/>
+      <x:c r="B71" s="12"/>
+      <x:c r="C71" s="12"/>
+    </x:row>
+    <x:row r="72" ht="28" customHeight="1">
+      <x:c r="A72" s="12"/>
+      <x:c r="B72" s="12"/>
+      <x:c r="C72" s="12"/>
+    </x:row>
+    <x:row r="73" ht="28" customHeight="1">
+      <x:c r="A73" s="12"/>
+      <x:c r="B73" s="12"/>
+      <x:c r="C73" s="12"/>
+    </x:row>
+    <x:row r="74" ht="28" customHeight="1">
+      <x:c r="A74" s="12"/>
+      <x:c r="B74" s="12"/>
+      <x:c r="C74" s="12"/>
+    </x:row>
+    <x:row r="75" ht="28" customHeight="1">
+      <x:c r="A75" s="12"/>
+      <x:c r="B75" s="12"/>
+      <x:c r="C75" s="12"/>
+    </x:row>
+    <x:row r="76" ht="28" customHeight="1">
+      <x:c r="A76" s="12"/>
+      <x:c r="B76" s="12"/>
+      <x:c r="C76" s="12"/>
+    </x:row>
+    <x:row r="77" ht="28" customHeight="1">
+      <x:c r="A77" s="12"/>
+      <x:c r="B77" s="12"/>
+      <x:c r="C77" s="12"/>
+    </x:row>
+    <x:row r="78" ht="28" customHeight="1">
+      <x:c r="A78" s="12"/>
+      <x:c r="B78" s="12"/>
+      <x:c r="C78" s="12"/>
+    </x:row>
+    <x:row r="79" ht="28" customHeight="1">
+      <x:c r="A79" s="12"/>
+      <x:c r="B79" s="12"/>
+      <x:c r="C79" s="12"/>
+    </x:row>
+    <x:row r="80" ht="28" customHeight="1">
+      <x:c r="A80" s="12"/>
+      <x:c r="B80" s="12"/>
+      <x:c r="C80" s="12"/>
+    </x:row>
+    <x:row r="81" ht="28" customHeight="1">
+      <x:c r="A81" s="12"/>
+      <x:c r="B81" s="12"/>
+      <x:c r="C81" s="12"/>
+    </x:row>
+    <x:row r="82" ht="28" customHeight="1">
+      <x:c r="A82" s="12"/>
+      <x:c r="B82" s="12"/>
+      <x:c r="C82" s="12"/>
+    </x:row>
+    <x:row r="83" ht="28" customHeight="1">
+      <x:c r="A83" s="12"/>
+      <x:c r="B83" s="12"/>
+      <x:c r="C83" s="12"/>
+    </x:row>
+    <x:row r="84" ht="28" customHeight="1">
+      <x:c r="A84" s="12"/>
+      <x:c r="B84" s="12"/>
+      <x:c r="C84" s="12"/>
+    </x:row>
+    <x:row r="85" ht="28" customHeight="1">
+      <x:c r="A85" s="12"/>
+      <x:c r="B85" s="12"/>
+      <x:c r="C85" s="12"/>
+    </x:row>
+    <x:row r="86" ht="28" customHeight="1">
+      <x:c r="A86" s="12"/>
+      <x:c r="B86" s="12"/>
+      <x:c r="C86" s="12"/>
+    </x:row>
+    <x:row r="87" ht="28" customHeight="1">
+      <x:c r="A87" s="12"/>
+      <x:c r="B87" s="12"/>
+      <x:c r="C87" s="12"/>
+    </x:row>
+    <x:row r="88" ht="28" customHeight="1">
+      <x:c r="A88" s="12"/>
+      <x:c r="B88" s="12"/>
+      <x:c r="C88" s="12"/>
+    </x:row>
+    <x:row r="89" ht="28" customHeight="1">
+      <x:c r="A89" s="12"/>
+      <x:c r="B89" s="12"/>
+      <x:c r="C89" s="12"/>
+    </x:row>
+    <x:row r="90" ht="28" customHeight="1">
+      <x:c r="A90" s="12"/>
+      <x:c r="B90" s="12"/>
+      <x:c r="C90" s="12"/>
+    </x:row>
+    <x:row r="91" ht="28" customHeight="1">
+      <x:c r="A91" s="12"/>
+      <x:c r="B91" s="12"/>
+      <x:c r="C91" s="12"/>
+    </x:row>
+    <x:row r="92" ht="28" customHeight="1">
+      <x:c r="A92" s="12"/>
+      <x:c r="B92" s="12"/>
+      <x:c r="C92" s="12"/>
+    </x:row>
+    <x:row r="93" ht="28" customHeight="1">
+      <x:c r="A93" s="12"/>
+      <x:c r="B93" s="12"/>
+      <x:c r="C93" s="12"/>
+    </x:row>
+    <x:row r="94" ht="28" customHeight="1">
+      <x:c r="A94" s="12"/>
+      <x:c r="B94" s="12"/>
+      <x:c r="C94" s="12"/>
+    </x:row>
+    <x:row r="95" ht="28" customHeight="1">
+      <x:c r="A95" s="12"/>
+      <x:c r="B95" s="12"/>
+      <x:c r="C95" s="12"/>
+    </x:row>
+    <x:row r="96" ht="28" customHeight="1">
+      <x:c r="A96" s="12"/>
+      <x:c r="B96" s="12"/>
+      <x:c r="C96" s="12"/>
+    </x:row>
+    <x:row r="97" ht="28" customHeight="1">
+      <x:c r="A97" s="12"/>
+      <x:c r="B97" s="12"/>
+      <x:c r="C97" s="12"/>
+    </x:row>
+    <x:row r="98" ht="28" customHeight="1">
+      <x:c r="A98" s="12"/>
+      <x:c r="B98" s="12"/>
+      <x:c r="C98" s="12"/>
+    </x:row>
+    <x:row r="99" ht="28" customHeight="1">
+      <x:c r="A99" s="12"/>
+      <x:c r="B99" s="12"/>
+      <x:c r="C99" s="12"/>
+    </x:row>
+    <x:row r="100" ht="28" customHeight="1">
+      <x:c r="A100" s="12"/>
+      <x:c r="B100" s="12"/>
+      <x:c r="C100" s="12"/>
+    </x:row>
+    <x:row r="101" ht="28" customHeight="1">
+      <x:c r="A101" s="12"/>
+      <x:c r="B101" s="12"/>
+      <x:c r="C101" s="12"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>